<commit_message>
Add Amasus classification and hierarchy PDF
</commit_message>
<xml_diff>
--- a/classification_familles_epr2.xlsx
+++ b/classification_familles_epr2.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Briese" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vertom" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAL" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amasus" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Briese'!$A$1:$P$42</definedName>
@@ -18,6 +19,8 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Vertom'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SAL'!$A$1:$P$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'SAL'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Amasus'!$A$1:$P$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Amasus'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -301,6 +304,31 @@
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SALFamilyTable" displayName="SALFamilyTable" ref="A1:P59" headerRowCount="1">
   <autoFilter ref="A1:P59"/>
+  <tableColumns count="16">
+    <tableColumn id="1" name="N°"/>
+    <tableColumn id="2" name="Famille"/>
+    <tableColumn id="3" name="Nom du bateau"/>
+    <tableColumn id="4" name="Type de navire"/>
+    <tableColumn id="5" name="Classe"/>
+    <tableColumn id="6" name="Nombre max de colis"/>
+    <tableColumn id="7" name="Longueur (m)"/>
+    <tableColumn id="8" name="Largeur (m)"/>
+    <tableColumn id="9" name="Tirant d’eau (m)"/>
+    <tableColumn id="10" name="Faisabilité de grue (Oui/Non)"/>
+    <tableColumn id="11" name="Note"/>
+    <tableColumn id="12" name="Nombre max de colis après limite de grue"/>
+    <tableColumn id="13" name="Deux grues nécessaires (Oui/Non)"/>
+    <tableColumn id="14" name="Priorité"/>
+    <tableColumn id="15" name="Navire sœur ? (Oui/Non)"/>
+    <tableColumn id="16" name="Lien PDF"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="AmasusFamilyTable" displayName="AmasusFamilyTable" ref="A1:P7" headerRowCount="1">
+  <autoFilter ref="A1:P7"/>
   <tableColumns count="16">
     <tableColumn id="1" name="N°"/>
     <tableColumn id="2" name="Famille"/>
@@ -9323,4 +9351,374 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="54" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Famille</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nom du bateau</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Type de navire</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre max de colis</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Longueur (m)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Largeur (m)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Tirant d’eau (m)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Faisabilité de grue (Oui/Non)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre max de colis après limite de grue</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Deux grues nécessaires (Oui/Non)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Navire sœur ? (Oui/Non)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Lien PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Eems Duisburg</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Eems Duisburg</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>NC (navire conventionnel)</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>CE–NC</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="n"/>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="9" t="n"/>
+      <c r="J2" s="9" t="n"/>
+      <c r="K2" s="9" t="n"/>
+      <c r="L2" s="9" t="n"/>
+      <c r="M2" s="9" t="n"/>
+      <c r="N2" s="9" t="n"/>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Polarrock</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Polarrock</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>NC (navire conventionnel)</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>CE–NC</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="n"/>
+      <c r="G3" s="11" t="n"/>
+      <c r="H3" s="11" t="n"/>
+      <c r="I3" s="11" t="n"/>
+      <c r="J3" s="11" t="n"/>
+      <c r="K3" s="11" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
+      <c r="N3" s="11" t="n"/>
+      <c r="O3" s="11" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="P3" s="11" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Eems Duisburg</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Eems Duisburg</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>NC (navire conventionnel)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>PP–NC</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="9" t="n"/>
+      <c r="J4" s="9" t="n"/>
+      <c r="K4" s="9" t="n"/>
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="9" t="n"/>
+      <c r="N4" s="9" t="n"/>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Polarrock</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Polarrock</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>NC (navire conventionnel)</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>PP–NC</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="n"/>
+      <c r="G5" s="11" t="n"/>
+      <c r="H5" s="11" t="n"/>
+      <c r="I5" s="11" t="n"/>
+      <c r="J5" s="11" t="n"/>
+      <c r="K5" s="11" t="n"/>
+      <c r="L5" s="11" t="n"/>
+      <c r="M5" s="11" t="n"/>
+      <c r="N5" s="11" t="n"/>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="P5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Eems Duisburg</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Eems Duisburg</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>NC (navire conventionnel)</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>GV–NC</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="9" t="n"/>
+      <c r="N6" s="9" t="n"/>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Polarrock</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Polarrock</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>NC (navire conventionnel)</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>GV–NC</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="11" t="n"/>
+      <c r="K7" s="11" t="n"/>
+      <c r="L7" s="11" t="n"/>
+      <c r="M7" s="11" t="n"/>
+      <c r="N7" s="11" t="n"/>
+      <c r="O7" s="11" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="P7" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P7">
+    <filterColumn colId="14" hiddenButton="0" showButton="1">
+      <filters blank="0">
+        <filter val="Non"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <dataValidations count="1">
+    <dataValidation sqref="J2:J7 M2:M7 O2:O7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Use MS prefixes for Amasus vessels
</commit_message>
<xml_diff>
--- a/classification_familles_epr2.xlsx
+++ b/classification_familles_epr2.xlsx
@@ -9473,7 +9473,7 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>Eems Duisburg</t>
+          <t>MS Eems Duisburg</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -9513,7 +9513,7 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>Polarrock</t>
+          <t>MS Polarrock</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
@@ -9553,7 +9553,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Eems Duisburg</t>
+          <t>MS Eems Duisburg</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -9593,7 +9593,7 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Polarrock</t>
+          <t>MS Polarrock</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
@@ -9633,7 +9633,7 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Eems Duisburg</t>
+          <t>MS Eems Duisburg</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -9673,7 +9673,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Polarrock</t>
+          <t>MS Polarrock</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">

</xml_diff>